<commit_message>
fix dépendance current -> latest 647cbb0e5d45854f19e939bdb2edb99ce9e41b09
</commit_message>
<xml_diff>
--- a/spec-tech/ig/StructureDefinition-pdlgcArchivePatient.xlsx
+++ b/spec-tech/ig/StructureDefinition-pdlgcArchivePatient.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-30T15:04:16+00:00</t>
+    <t>2026-08-07T08:28:26+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -379,37 +379,37 @@
     <t>Document PDF destiné à la consultation. Ces documents ne sont pas intégrés par le destinataire si le destinataire est une système.</t>
   </si>
   <si>
-    <t>pdlgcArchivePatient.iheXdm</t>
+    <t>pdlgcArchivePatient.iheXDM</t>
   </si>
   <si>
     <t>répertoire IHE_XDM contenant le lot de soumissions des données d'un patient. Nom du répertoire fixé à IHE_XDM.</t>
   </si>
   <si>
-    <t>pdlgcArchivePatient.iheXdm.id</t>
-  </si>
-  <si>
-    <t>pdlgcArchivePatient.iheXdm.extension</t>
-  </si>
-  <si>
-    <t>pdlgcArchivePatient.iheXdm.modifierExtension</t>
-  </si>
-  <si>
-    <t>pdlgcArchivePatient.iheXdm.subset01</t>
+    <t>pdlgcArchivePatient.iheXDM.id</t>
+  </si>
+  <si>
+    <t>pdlgcArchivePatient.iheXDM.extension</t>
+  </si>
+  <si>
+    <t>pdlgcArchivePatient.iheXDM.modifierExtension</t>
+  </si>
+  <si>
+    <t>pdlgcArchivePatient.iheXDM.subset01</t>
   </si>
   <si>
     <t>lot de soumission contenant les données d'un patient.</t>
   </si>
   <si>
-    <t>pdlgcArchivePatient.iheXdm.subset01.id</t>
-  </si>
-  <si>
-    <t>pdlgcArchivePatient.iheXdm.subset01.extension</t>
-  </si>
-  <si>
-    <t>pdlgcArchivePatient.iheXdm.subset01.modifierExtension</t>
-  </si>
-  <si>
-    <t>pdlgcArchivePatient.iheXdm.subset01.metadata</t>
+    <t>pdlgcArchivePatient.iheXDM.subset01.id</t>
+  </si>
+  <si>
+    <t>pdlgcArchivePatient.iheXDM.subset01.extension</t>
+  </si>
+  <si>
+    <t>pdlgcArchivePatient.iheXDM.subset01.modifierExtension</t>
+  </si>
+  <si>
+    <t>pdlgcArchivePatient.iheXDM.subset01.metadata</t>
   </si>
   <si>
     <t xml:space="preserve">https://interop.esante.gouv.fr/ig/fhir/pdlgc/StructureDefinition/pdlgcMetadata
@@ -419,13 +419,13 @@
     <t>métadonnées du lot de soumission, conforme au profil IHE XDM, décrivant les documents patient qu'il accompagne.</t>
   </si>
   <si>
-    <t>pdlgcArchivePatient.iheXdm.subset01.documentPivot</t>
+    <t>pdlgcArchivePatient.iheXDM.subset01.documentPivot</t>
   </si>
   <si>
     <t>Données structurées du périmètres pivot, concernant les informations administratives et médicales du patient. Leur export est obligatoire.</t>
   </si>
   <si>
-    <t>pdlgcArchivePatient.iheXdm.subset01.documentHorsPivot</t>
+    <t>pdlgcArchivePatient.iheXDM.subset01.documentHorsPivot</t>
   </si>
   <si>
     <t>Données structurées hors périmètre pivot. Leur export est facultatif.</t>
@@ -733,8 +733,8 @@
   <dimension ref="A1:AJ20"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="46.796875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="46.796875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="46.8359375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="46.8359375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="18.19140625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -764,7 +764,7 @@
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="46.796875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="46.8359375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>

</xml_diff>